<commit_message>
docs: update runtime modifiable parameters Excel files
</commit_message>
<xml_diff>
--- a/docs/en/source/_static/files/runtime_modifiable_parameters.xlsx
+++ b/docs/en/source/_static/files/runtime_modifiable_parameters.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="881" uniqueCount="496">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="925" uniqueCount="495">
   <si>
     <t>ID</t>
   </si>
@@ -48,7 +48,7 @@
 (336/336L)</t>
   </si>
   <si>
-    <t>Range (336L)</t>
+    <t xml:space="preserve">Range </t>
   </si>
   <si>
     <t>ROS get</t>
@@ -72,7 +72,7 @@
     <t>R/W</t>
   </si>
   <si>
-    <t>WO</t>
+    <t>_/W</t>
   </si>
   <si>
     <t>Bool value(min:0, max:1, step:1)</t>
@@ -126,6 +126,9 @@
     <t>Enable/disable temperature compensation   *</t>
   </si>
   <si>
+    <t>_/_</t>
+  </si>
+  <si>
     <t>OB_PROP_DEPTH_MIRROR_BOOL</t>
   </si>
   <si>
@@ -207,9 +210,6 @@
     <t>R/_</t>
   </si>
   <si>
-    <t>RO</t>
-  </si>
-  <si>
     <t>service: get_ldp_status</t>
   </si>
   <si>
@@ -408,9 +408,6 @@
     <t>Reset device time to zero</t>
   </si>
   <si>
-    <t>_/W</t>
-  </si>
-  <si>
     <t>OB_PROP_TIMER_RESET_TRIGGER_OUT_ENABLE_BOOL</t>
   </si>
   <si>
@@ -594,6 +591,9 @@
     <t>Laser on/off alternate mode, 0: off, 1: on-off alternate, 2: off-on alternate</t>
   </si>
   <si>
+    <t>OB_PROP_DEPTH_UNIT_FLEXIBLE_ADJUSTMENT_FLOAT</t>
+  </si>
+  <si>
     <t>Depth unit flexible adjustment\</t>
   </si>
   <si>
@@ -718,9 +718,6 @@
   </si>
   <si>
     <t>Get the health check result from device,range is [0.0f,1.5f]</t>
-  </si>
-  <si>
-    <t>Float value(min:0.000000, max:0.000000, step:0.000000)</t>
   </si>
   <si>
     <t>OB_PROP_ON_CHIP_CALIBRATION_ENABLE_BOOL</t>
@@ -2834,6 +2831,9 @@
       <c r="E8" t="s">
         <v>13</v>
       </c>
+      <c r="F8" t="s">
+        <v>32</v>
+      </c>
       <c r="G8" t="s">
         <v>15</v>
       </c>
@@ -2843,13 +2843,13 @@
         <v>14</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C9" t="s">
         <v>11</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E9" t="s">
         <v>13</v>
@@ -2864,7 +2864,7 @@
         <v>16</v>
       </c>
       <c r="I9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -2872,13 +2872,13 @@
         <v>15</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C10" t="s">
         <v>11</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E10" t="s">
         <v>13</v>
@@ -2893,7 +2893,7 @@
         <v>16</v>
       </c>
       <c r="I10" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:10">
@@ -2901,13 +2901,13 @@
         <v>16</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C11" t="s">
         <v>11</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12" spans="1:10">
@@ -2915,13 +2915,13 @@
         <v>17</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C12" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="13" spans="1:10">
@@ -2929,13 +2929,13 @@
         <v>18</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C13" t="s">
         <v>11</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E13" t="s">
         <v>13</v>
@@ -2950,7 +2950,7 @@
         <v>16</v>
       </c>
       <c r="I13" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="14" spans="1:10">
@@ -2958,13 +2958,13 @@
         <v>19</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C14" t="s">
         <v>11</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E14" t="s">
         <v>13</v>
@@ -2979,7 +2979,7 @@
         <v>16</v>
       </c>
       <c r="I14" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:10">
@@ -2987,13 +2987,13 @@
         <v>22</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C15" t="s">
         <v>21</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16" spans="1:10">
@@ -3001,13 +3001,13 @@
         <v>23</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C16" t="s">
         <v>21</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -3015,13 +3015,13 @@
         <v>24</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C17" t="s">
         <v>11</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E17" t="s">
         <v>13</v>
@@ -3033,10 +3033,10 @@
         <v>15</v>
       </c>
       <c r="H17" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I17" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -3044,16 +3044,16 @@
         <v>32</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C18" t="s">
         <v>11</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E18" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F18" t="s">
         <v>59</v>
@@ -3088,10 +3088,10 @@
         <v>13</v>
       </c>
       <c r="H19" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I19" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="20" ht="36" spans="1:9">
@@ -3114,10 +3114,10 @@
         <v>13</v>
       </c>
       <c r="H20" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I20" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="21" spans="1:9">
@@ -3136,6 +3136,9 @@
       <c r="E21" t="s">
         <v>13</v>
       </c>
+      <c r="F21" t="s">
+        <v>32</v>
+      </c>
       <c r="G21" t="s">
         <v>15</v>
       </c>
@@ -3354,6 +3357,9 @@
       <c r="E34" t="s">
         <v>13</v>
       </c>
+      <c r="F34" t="s">
+        <v>32</v>
+      </c>
       <c r="G34" t="s">
         <v>15</v>
       </c>
@@ -3402,6 +3408,9 @@
       <c r="E37" t="s">
         <v>13</v>
       </c>
+      <c r="F37" t="s">
+        <v>32</v>
+      </c>
       <c r="G37" t="s">
         <v>15</v>
       </c>
@@ -3422,6 +3431,9 @@
       <c r="E38" t="s">
         <v>13</v>
       </c>
+      <c r="F38" t="s">
+        <v>32</v>
+      </c>
       <c r="G38" t="s">
         <v>15</v>
       </c>
@@ -3540,6 +3552,9 @@
       <c r="E46" t="s">
         <v>13</v>
       </c>
+      <c r="F46" t="s">
+        <v>32</v>
+      </c>
       <c r="G46" t="s">
         <v>119</v>
       </c>
@@ -3558,7 +3573,7 @@
         <v>121</v>
       </c>
       <c r="E47" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F47" t="s">
         <v>59</v>
@@ -3587,7 +3602,10 @@
         <v>125</v>
       </c>
       <c r="E48" t="s">
-        <v>126</v>
+        <v>14</v>
+      </c>
+      <c r="F48" t="s">
+        <v>32</v>
       </c>
       <c r="G48" t="s">
         <v>15</v>
@@ -3598,16 +3616,19 @@
         <v>105</v>
       </c>
       <c r="B49" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C49" t="s">
+        <v>11</v>
+      </c>
+      <c r="D49" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="C49" t="s">
-        <v>11</v>
-      </c>
-      <c r="D49" s="1" t="s">
-        <v>128</v>
-      </c>
       <c r="E49" t="s">
         <v>13</v>
+      </c>
+      <c r="F49" t="s">
+        <v>32</v>
       </c>
       <c r="G49" t="s">
         <v>15</v>
@@ -3618,19 +3639,22 @@
         <v>106</v>
       </c>
       <c r="B50" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C50" t="s">
+        <v>21</v>
+      </c>
+      <c r="D50" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="C50" t="s">
-        <v>21</v>
-      </c>
-      <c r="D50" s="1" t="s">
+      <c r="E50" t="s">
+        <v>13</v>
+      </c>
+      <c r="F50" t="s">
+        <v>32</v>
+      </c>
+      <c r="G50" t="s">
         <v>130</v>
-      </c>
-      <c r="E50" t="s">
-        <v>13</v>
-      </c>
-      <c r="G50" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="51" spans="1:9">
@@ -3638,16 +3662,19 @@
         <v>107</v>
       </c>
       <c r="B51" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C51" t="s">
+        <v>11</v>
+      </c>
+      <c r="D51" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="C51" t="s">
-        <v>11</v>
-      </c>
-      <c r="D51" s="1" t="s">
-        <v>133</v>
-      </c>
       <c r="E51" t="s">
-        <v>126</v>
+        <v>14</v>
+      </c>
+      <c r="F51" t="s">
+        <v>32</v>
       </c>
       <c r="G51" t="s">
         <v>15</v>
@@ -3658,13 +3685,13 @@
         <v>112</v>
       </c>
       <c r="B52" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C52" t="s">
+        <v>11</v>
+      </c>
+      <c r="D52" s="1" t="s">
         <v>134</v>
-      </c>
-      <c r="C52" t="s">
-        <v>11</v>
-      </c>
-      <c r="D52" s="1" t="s">
-        <v>135</v>
       </c>
       <c r="E52" t="s">
         <v>13</v>
@@ -3679,7 +3706,7 @@
         <v>16</v>
       </c>
       <c r="I52" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="53" ht="54" spans="1:9">
@@ -3687,19 +3714,22 @@
         <v>113</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C53" t="s">
         <v>11</v>
       </c>
       <c r="D53" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="E53" t="s">
+        <v>13</v>
+      </c>
+      <c r="F53" t="s">
+        <v>32</v>
+      </c>
+      <c r="G53" t="s">
         <v>137</v>
-      </c>
-      <c r="E53" t="s">
-        <v>13</v>
-      </c>
-      <c r="G53" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="54" ht="36" spans="1:9">
@@ -3707,13 +3737,13 @@
         <v>114</v>
       </c>
       <c r="B54" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="C54" t="s">
+        <v>11</v>
+      </c>
+      <c r="D54" s="1" t="s">
         <v>139</v>
-      </c>
-      <c r="C54" t="s">
-        <v>11</v>
-      </c>
-      <c r="D54" s="1" t="s">
-        <v>140</v>
       </c>
       <c r="E54" t="s">
         <v>13</v>
@@ -3728,7 +3758,7 @@
         <v>16</v>
       </c>
       <c r="I54" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="55" spans="1:9">
@@ -3736,13 +3766,13 @@
         <v>115</v>
       </c>
       <c r="B55" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="C55" t="s">
+        <v>21</v>
+      </c>
+      <c r="D55" s="1" t="s">
         <v>142</v>
-      </c>
-      <c r="C55" t="s">
-        <v>21</v>
-      </c>
-      <c r="D55" s="1" t="s">
-        <v>143</v>
       </c>
       <c r="E55" t="s">
         <v>13</v>
@@ -3754,7 +3784,7 @@
         <v>16</v>
       </c>
       <c r="I55" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="56" spans="1:9">
@@ -3762,13 +3792,13 @@
         <v>116</v>
       </c>
       <c r="B56" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="C56" t="s">
+        <v>21</v>
+      </c>
+      <c r="D56" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="C56" t="s">
-        <v>21</v>
-      </c>
-      <c r="D56" s="1" t="s">
-        <v>146</v>
       </c>
       <c r="E56" t="s">
         <v>13</v>
@@ -3780,7 +3810,7 @@
         <v>16</v>
       </c>
       <c r="I56" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="57" spans="1:9">
@@ -3788,13 +3818,13 @@
         <v>117</v>
       </c>
       <c r="B57" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="C57" t="s">
+        <v>21</v>
+      </c>
+      <c r="D57" s="1" t="s">
         <v>148</v>
-      </c>
-      <c r="C57" t="s">
-        <v>21</v>
-      </c>
-      <c r="D57" s="1" t="s">
-        <v>149</v>
       </c>
       <c r="E57" t="s">
         <v>13</v>
@@ -3806,7 +3836,7 @@
         <v>16</v>
       </c>
       <c r="I57" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="58" spans="1:9">
@@ -3814,13 +3844,13 @@
         <v>118</v>
       </c>
       <c r="B58" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="C58" t="s">
+        <v>21</v>
+      </c>
+      <c r="D58" s="1" t="s">
         <v>151</v>
-      </c>
-      <c r="C58" t="s">
-        <v>21</v>
-      </c>
-      <c r="D58" s="1" t="s">
-        <v>152</v>
       </c>
       <c r="E58" t="s">
         <v>13</v>
@@ -3832,7 +3862,7 @@
         <v>16</v>
       </c>
       <c r="I58" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="59" ht="90" spans="1:9">
@@ -3840,16 +3870,19 @@
         <v>119</v>
       </c>
       <c r="B59" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="C59" t="s">
+        <v>21</v>
+      </c>
+      <c r="D59" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="C59" t="s">
-        <v>21</v>
-      </c>
-      <c r="D59" s="1" t="s">
-        <v>155</v>
-      </c>
       <c r="E59" t="s">
-        <v>58</v>
+        <v>59</v>
+      </c>
+      <c r="F59" t="s">
+        <v>32</v>
       </c>
       <c r="G59" t="s">
         <v>119</v>
@@ -3860,13 +3893,13 @@
         <v>121</v>
       </c>
       <c r="B60" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="C60" t="s">
+        <v>21</v>
+      </c>
+      <c r="D60" s="1" t="s">
         <v>156</v>
-      </c>
-      <c r="C60" t="s">
-        <v>21</v>
-      </c>
-      <c r="D60" s="1" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="61" spans="1:9">
@@ -3874,13 +3907,13 @@
         <v>122</v>
       </c>
       <c r="B61" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="C61" t="s">
+        <v>21</v>
+      </c>
+      <c r="D61" s="1" t="s">
         <v>158</v>
-      </c>
-      <c r="C61" t="s">
-        <v>21</v>
-      </c>
-      <c r="D61" s="1" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="62" ht="54" spans="1:9">
@@ -3888,13 +3921,13 @@
         <v>129</v>
       </c>
       <c r="B62" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="C62" t="s">
+        <v>21</v>
+      </c>
+      <c r="D62" s="1" t="s">
         <v>160</v>
-      </c>
-      <c r="C62" t="s">
-        <v>21</v>
-      </c>
-      <c r="D62" s="1" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="63" ht="36" spans="1:9">
@@ -3902,16 +3935,19 @@
         <v>130</v>
       </c>
       <c r="B63" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="C63" t="s">
+        <v>11</v>
+      </c>
+      <c r="D63" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="C63" t="s">
-        <v>11</v>
-      </c>
-      <c r="D63" s="1" t="s">
-        <v>163</v>
-      </c>
       <c r="E63" t="s">
         <v>13</v>
+      </c>
+      <c r="F63" t="s">
+        <v>32</v>
       </c>
       <c r="G63" t="s">
         <v>15</v>
@@ -3922,13 +3958,13 @@
         <v>131</v>
       </c>
       <c r="B64" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="C64" t="s">
+        <v>11</v>
+      </c>
+      <c r="D64" s="1" t="s">
         <v>164</v>
-      </c>
-      <c r="C64" t="s">
-        <v>11</v>
-      </c>
-      <c r="D64" s="1" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="65" spans="1:9">
@@ -3936,13 +3972,13 @@
         <v>132</v>
       </c>
       <c r="B65" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="C65" t="s">
+        <v>11</v>
+      </c>
+      <c r="D65" s="1" t="s">
         <v>166</v>
-      </c>
-      <c r="C65" t="s">
-        <v>11</v>
-      </c>
-      <c r="D65" s="1" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="66" ht="36" spans="1:9">
@@ -3950,13 +3986,13 @@
         <v>133</v>
       </c>
       <c r="B66" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C66" t="s">
+        <v>11</v>
+      </c>
+      <c r="D66" s="1" t="s">
         <v>168</v>
-      </c>
-      <c r="C66" t="s">
-        <v>11</v>
-      </c>
-      <c r="D66" s="1" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="67" spans="1:9">
@@ -3964,13 +4000,13 @@
         <v>134</v>
       </c>
       <c r="B67" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="C67" t="s">
+        <v>21</v>
+      </c>
+      <c r="D67" s="1" t="s">
         <v>170</v>
-      </c>
-      <c r="C67" t="s">
-        <v>21</v>
-      </c>
-      <c r="D67" s="1" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="68" spans="1:9">
@@ -3978,13 +4014,13 @@
         <v>135</v>
       </c>
       <c r="B68" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="C68" t="s">
+        <v>21</v>
+      </c>
+      <c r="D68" s="1" t="s">
         <v>172</v>
-      </c>
-      <c r="C68" t="s">
-        <v>21</v>
-      </c>
-      <c r="D68" s="1" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="69" spans="1:9">
@@ -3992,13 +4028,13 @@
         <v>136</v>
       </c>
       <c r="B69" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="C69" t="s">
+        <v>21</v>
+      </c>
+      <c r="D69" s="1" t="s">
         <v>174</v>
-      </c>
-      <c r="C69" t="s">
-        <v>21</v>
-      </c>
-      <c r="D69" s="1" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="70" ht="54" spans="1:9">
@@ -4006,16 +4042,19 @@
         <v>141</v>
       </c>
       <c r="B70" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="C70" t="s">
+        <v>11</v>
+      </c>
+      <c r="D70" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="C70" t="s">
-        <v>11</v>
-      </c>
-      <c r="D70" s="1" t="s">
-        <v>177</v>
-      </c>
       <c r="E70" t="s">
         <v>13</v>
+      </c>
+      <c r="F70" t="s">
+        <v>32</v>
       </c>
       <c r="G70" t="s">
         <v>15</v>
@@ -4026,13 +4065,13 @@
         <v>142</v>
       </c>
       <c r="B71" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="C71" t="s">
+        <v>21</v>
+      </c>
+      <c r="D71" s="1" t="s">
         <v>178</v>
-      </c>
-      <c r="C71" t="s">
-        <v>21</v>
-      </c>
-      <c r="D71" s="1" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="72" ht="36" spans="1:9">
@@ -4040,13 +4079,13 @@
         <v>148</v>
       </c>
       <c r="B72" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="C72" t="s">
+        <v>11</v>
+      </c>
+      <c r="D72" s="1" t="s">
         <v>180</v>
-      </c>
-      <c r="C72" t="s">
-        <v>11</v>
-      </c>
-      <c r="D72" s="1" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="73" ht="36" spans="1:9">
@@ -4054,13 +4093,13 @@
         <v>149</v>
       </c>
       <c r="B73" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="C73" t="s">
+        <v>11</v>
+      </c>
+      <c r="D73" s="1" t="s">
         <v>182</v>
-      </c>
-      <c r="C73" t="s">
-        <v>11</v>
-      </c>
-      <c r="D73" s="1" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="74" ht="36" spans="1:9">
@@ -4068,16 +4107,19 @@
         <v>174</v>
       </c>
       <c r="B74" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="C74" t="s">
+        <v>11</v>
+      </c>
+      <c r="D74" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="C74" t="s">
-        <v>11</v>
-      </c>
-      <c r="D74" s="1" t="s">
-        <v>185</v>
-      </c>
       <c r="E74" t="s">
         <v>13</v>
+      </c>
+      <c r="F74" t="s">
+        <v>32</v>
       </c>
       <c r="G74" t="s">
         <v>15</v>
@@ -4088,36 +4130,42 @@
         <v>175</v>
       </c>
       <c r="B75" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="C75" t="s">
+        <v>21</v>
+      </c>
+      <c r="D75" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="C75" t="s">
-        <v>21</v>
-      </c>
-      <c r="D75" s="1" t="s">
-        <v>187</v>
-      </c>
       <c r="E75" t="s">
         <v>13</v>
+      </c>
+      <c r="F75" t="s">
+        <v>32</v>
       </c>
       <c r="G75" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="76" spans="1:9">
+    <row r="76" ht="36" spans="1:9">
       <c r="A76">
         <v>176</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>77</v>
+        <v>187</v>
       </c>
       <c r="C76" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D76" s="1" t="s">
         <v>188</v>
       </c>
       <c r="E76" t="s">
         <v>13</v>
+      </c>
+      <c r="F76" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="77" spans="1:9">
@@ -4165,6 +4213,9 @@
       <c r="E78" t="s">
         <v>13</v>
       </c>
+      <c r="F78" t="s">
+        <v>32</v>
+      </c>
       <c r="G78" t="s">
         <v>196</v>
       </c>
@@ -4183,7 +4234,10 @@
         <v>198</v>
       </c>
       <c r="E79" t="s">
-        <v>58</v>
+        <v>59</v>
+      </c>
+      <c r="F79" t="s">
+        <v>32</v>
       </c>
       <c r="G79" t="s">
         <v>15</v>
@@ -4205,6 +4259,9 @@
       <c r="E80" t="s">
         <v>13</v>
       </c>
+      <c r="F80" t="s">
+        <v>32</v>
+      </c>
       <c r="G80" t="s">
         <v>201</v>
       </c>
@@ -4225,6 +4282,9 @@
       <c r="E81" t="s">
         <v>13</v>
       </c>
+      <c r="F81" t="s">
+        <v>32</v>
+      </c>
       <c r="G81" t="s">
         <v>204</v>
       </c>
@@ -4345,6 +4405,9 @@
       <c r="E87" t="s">
         <v>13</v>
       </c>
+      <c r="F87" t="s">
+        <v>32</v>
+      </c>
       <c r="G87" t="s">
         <v>15</v>
       </c>
@@ -4379,6 +4442,9 @@
       <c r="E89" t="s">
         <v>13</v>
       </c>
+      <c r="F89" t="s">
+        <v>32</v>
+      </c>
       <c r="G89" t="s">
         <v>122</v>
       </c>
@@ -4399,6 +4465,9 @@
       <c r="E90" t="s">
         <v>13</v>
       </c>
+      <c r="F90" t="s">
+        <v>32</v>
+      </c>
       <c r="G90" t="s">
         <v>15</v>
       </c>
@@ -4419,6 +4488,9 @@
       <c r="E91" t="s">
         <v>13</v>
       </c>
+      <c r="F91" t="s">
+        <v>32</v>
+      </c>
       <c r="G91" t="s">
         <v>122</v>
       </c>
@@ -4437,10 +4509,10 @@
         <v>229</v>
       </c>
       <c r="E92" t="s">
-        <v>58</v>
-      </c>
-      <c r="G92" t="s">
-        <v>230</v>
+        <v>59</v>
+      </c>
+      <c r="F92" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="93" spans="1:9">
@@ -4448,16 +4520,19 @@
         <v>210</v>
       </c>
       <c r="B93" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="C93" t="s">
+        <v>11</v>
+      </c>
+      <c r="D93" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="C93" t="s">
-        <v>11</v>
-      </c>
-      <c r="D93" s="1" t="s">
-        <v>232</v>
-      </c>
       <c r="E93" t="s">
         <v>13</v>
+      </c>
+      <c r="F93" t="s">
+        <v>32</v>
       </c>
       <c r="G93" t="s">
         <v>15</v>
@@ -4468,13 +4543,13 @@
         <v>211</v>
       </c>
       <c r="B94" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="C94" t="s">
+        <v>11</v>
+      </c>
+      <c r="D94" s="1" t="s">
         <v>233</v>
-      </c>
-      <c r="C94" t="s">
-        <v>11</v>
-      </c>
-      <c r="D94" s="1" t="s">
-        <v>234</v>
       </c>
       <c r="E94" t="s">
         <v>13</v>
@@ -4486,10 +4561,10 @@
         <v>15</v>
       </c>
       <c r="H94" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I94" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="95" ht="36" spans="1:9">
@@ -4497,28 +4572,28 @@
         <v>212</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C95" t="s">
         <v>24</v>
       </c>
       <c r="D95" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="E95" t="s">
+        <v>13</v>
+      </c>
+      <c r="F95" t="s">
+        <v>13</v>
+      </c>
+      <c r="G95" t="s">
         <v>236</v>
       </c>
-      <c r="E95" t="s">
-        <v>13</v>
-      </c>
-      <c r="F95" t="s">
-        <v>13</v>
-      </c>
-      <c r="G95" t="s">
-        <v>237</v>
-      </c>
       <c r="H95" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="I95" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="96" ht="54" spans="1:9">
@@ -4526,16 +4601,19 @@
         <v>216</v>
       </c>
       <c r="B96" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="C96" t="s">
+        <v>11</v>
+      </c>
+      <c r="D96" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="C96" t="s">
-        <v>11</v>
-      </c>
-      <c r="D96" s="1" t="s">
-        <v>239</v>
-      </c>
       <c r="E96" t="s">
         <v>13</v>
+      </c>
+      <c r="F96" t="s">
+        <v>32</v>
       </c>
       <c r="G96" t="s">
         <v>15</v>
@@ -4546,19 +4624,22 @@
         <v>217</v>
       </c>
       <c r="B97" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="C97" t="s">
+        <v>21</v>
+      </c>
+      <c r="D97" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="C97" t="s">
-        <v>11</v>
-      </c>
-      <c r="D97" s="1" t="s">
+      <c r="E97" t="s">
+        <v>13</v>
+      </c>
+      <c r="F97" t="s">
+        <v>32</v>
+      </c>
+      <c r="G97" t="s">
         <v>241</v>
-      </c>
-      <c r="E97" t="s">
-        <v>13</v>
-      </c>
-      <c r="G97" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="98" spans="1:7">
@@ -4566,13 +4647,13 @@
         <v>223</v>
       </c>
       <c r="B98" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="C98" t="s">
+        <v>11</v>
+      </c>
+      <c r="D98" s="1" t="s">
         <v>243</v>
-      </c>
-      <c r="C98" t="s">
-        <v>11</v>
-      </c>
-      <c r="D98" s="1" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="99" ht="36" spans="1:7">
@@ -4580,13 +4661,13 @@
         <v>224</v>
       </c>
       <c r="B99" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="C99" t="s">
+        <v>11</v>
+      </c>
+      <c r="D99" s="1" t="s">
         <v>245</v>
-      </c>
-      <c r="C99" t="s">
-        <v>11</v>
-      </c>
-      <c r="D99" s="1" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="100" spans="1:7">
@@ -4594,13 +4675,13 @@
         <v>226</v>
       </c>
       <c r="B100" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="C100" t="s">
+        <v>11</v>
+      </c>
+      <c r="D100" s="1" t="s">
         <v>247</v>
-      </c>
-      <c r="C100" t="s">
-        <v>11</v>
-      </c>
-      <c r="D100" s="1" t="s">
-        <v>248</v>
       </c>
     </row>
     <row r="101" ht="36" spans="1:7">
@@ -4608,13 +4689,13 @@
         <v>227</v>
       </c>
       <c r="B101" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="C101" t="s">
+        <v>21</v>
+      </c>
+      <c r="D101" s="1" t="s">
         <v>249</v>
-      </c>
-      <c r="C101" t="s">
-        <v>21</v>
-      </c>
-      <c r="D101" s="1" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="102" spans="1:7">
@@ -4622,13 +4703,13 @@
         <v>229</v>
       </c>
       <c r="B102" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="C102" t="s">
+        <v>11</v>
+      </c>
+      <c r="D102" s="1" t="s">
         <v>251</v>
-      </c>
-      <c r="C102" t="s">
-        <v>11</v>
-      </c>
-      <c r="D102" s="1" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="103" spans="1:7">
@@ -4636,13 +4717,13 @@
         <v>230</v>
       </c>
       <c r="B103" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="C103" t="s">
+        <v>11</v>
+      </c>
+      <c r="D103" s="1" t="s">
         <v>253</v>
-      </c>
-      <c r="C103" t="s">
-        <v>11</v>
-      </c>
-      <c r="D103" s="1" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="104" spans="1:7">
@@ -4650,13 +4731,13 @@
         <v>231</v>
       </c>
       <c r="B104" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="C104" t="s">
+        <v>21</v>
+      </c>
+      <c r="D104" s="1" t="s">
         <v>255</v>
-      </c>
-      <c r="C104" t="s">
-        <v>21</v>
-      </c>
-      <c r="D104" s="1" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="105" ht="54" spans="1:7">
@@ -4664,16 +4745,19 @@
         <v>236</v>
       </c>
       <c r="B105" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="C105" t="s">
+        <v>21</v>
+      </c>
+      <c r="D105" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="C105" t="s">
-        <v>21</v>
-      </c>
-      <c r="D105" s="1" t="s">
-        <v>258</v>
-      </c>
       <c r="E105" t="s">
         <v>13</v>
+      </c>
+      <c r="F105" t="s">
+        <v>32</v>
       </c>
       <c r="G105" t="s">
         <v>191</v>
@@ -4684,13 +4768,13 @@
         <v>242</v>
       </c>
       <c r="B106" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="C106" t="s">
+        <v>21</v>
+      </c>
+      <c r="D106" s="1" t="s">
         <v>259</v>
-      </c>
-      <c r="C106" t="s">
-        <v>21</v>
-      </c>
-      <c r="D106" s="1" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="107" spans="1:7">
@@ -4698,13 +4782,13 @@
         <v>243</v>
       </c>
       <c r="B107" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="C107" t="s">
+        <v>11</v>
+      </c>
+      <c r="D107" s="1" t="s">
         <v>261</v>
-      </c>
-      <c r="C107" t="s">
-        <v>11</v>
-      </c>
-      <c r="D107" s="1" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="108" spans="1:7">
@@ -4712,13 +4796,13 @@
         <v>244</v>
       </c>
       <c r="B108" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="C108" t="s">
+        <v>11</v>
+      </c>
+      <c r="D108" s="1" t="s">
         <v>263</v>
-      </c>
-      <c r="C108" t="s">
-        <v>11</v>
-      </c>
-      <c r="D108" s="1" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="109" ht="36" spans="1:7">
@@ -4726,13 +4810,13 @@
         <v>247</v>
       </c>
       <c r="B109" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="C109" t="s">
+        <v>21</v>
+      </c>
+      <c r="D109" s="1" t="s">
         <v>265</v>
-      </c>
-      <c r="C109" t="s">
-        <v>21</v>
-      </c>
-      <c r="D109" s="1" t="s">
-        <v>266</v>
       </c>
     </row>
     <row r="110" spans="1:7">
@@ -4740,13 +4824,13 @@
         <v>248</v>
       </c>
       <c r="B110" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="C110" t="s">
+        <v>21</v>
+      </c>
+      <c r="D110" s="1" t="s">
         <v>267</v>
-      </c>
-      <c r="C110" t="s">
-        <v>21</v>
-      </c>
-      <c r="D110" s="1" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="111" spans="1:7">
@@ -4754,13 +4838,13 @@
         <v>249</v>
       </c>
       <c r="B111" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="C111" t="s">
+        <v>21</v>
+      </c>
+      <c r="D111" s="1" t="s">
         <v>269</v>
-      </c>
-      <c r="C111" t="s">
-        <v>21</v>
-      </c>
-      <c r="D111" s="1" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="112" spans="1:7">
@@ -4768,13 +4852,13 @@
         <v>251</v>
       </c>
       <c r="B112" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="C112" t="s">
+        <v>21</v>
+      </c>
+      <c r="D112" s="1" t="s">
         <v>271</v>
-      </c>
-      <c r="C112" t="s">
-        <v>21</v>
-      </c>
-      <c r="D112" s="1" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="113" spans="1:7">
@@ -4782,13 +4866,13 @@
         <v>252</v>
       </c>
       <c r="B113" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="C113" t="s">
+        <v>11</v>
+      </c>
+      <c r="D113" s="1" t="s">
         <v>273</v>
-      </c>
-      <c r="C113" t="s">
-        <v>11</v>
-      </c>
-      <c r="D113" s="1" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="114" spans="1:7">
@@ -4796,13 +4880,13 @@
         <v>253</v>
       </c>
       <c r="B114" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="C114" t="s">
+        <v>11</v>
+      </c>
+      <c r="D114" s="1" t="s">
         <v>275</v>
-      </c>
-      <c r="C114" t="s">
-        <v>11</v>
-      </c>
-      <c r="D114" s="1" t="s">
-        <v>276</v>
       </c>
     </row>
     <row r="115" spans="1:7">
@@ -4810,16 +4894,19 @@
         <v>255</v>
       </c>
       <c r="B115" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="C115" t="s">
+        <v>21</v>
+      </c>
+      <c r="D115" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="C115" t="s">
-        <v>21</v>
-      </c>
-      <c r="D115" s="1" t="s">
-        <v>278</v>
-      </c>
       <c r="E115" t="s">
         <v>13</v>
+      </c>
+      <c r="F115" t="s">
+        <v>32</v>
       </c>
       <c r="G115" t="s">
         <v>122</v>
@@ -4830,13 +4917,13 @@
         <v>257</v>
       </c>
       <c r="B116" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="C116" t="s">
+        <v>11</v>
+      </c>
+      <c r="D116" s="1" t="s">
         <v>279</v>
-      </c>
-      <c r="C116" t="s">
-        <v>11</v>
-      </c>
-      <c r="D116" s="1" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="117" spans="1:7">
@@ -4844,13 +4931,13 @@
         <v>259</v>
       </c>
       <c r="B117" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="C117" t="s">
+        <v>11</v>
+      </c>
+      <c r="D117" s="1" t="s">
         <v>281</v>
-      </c>
-      <c r="C117" t="s">
-        <v>11</v>
-      </c>
-      <c r="D117" s="1" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="118" spans="1:7">
@@ -4858,13 +4945,13 @@
         <v>260</v>
       </c>
       <c r="B118" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="C118" t="s">
+        <v>21</v>
+      </c>
+      <c r="D118" s="1" t="s">
         <v>283</v>
-      </c>
-      <c r="C118" t="s">
-        <v>21</v>
-      </c>
-      <c r="D118" s="1" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="119" spans="1:7">
@@ -4872,13 +4959,13 @@
         <v>261</v>
       </c>
       <c r="B119" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="C119" t="s">
+        <v>21</v>
+      </c>
+      <c r="D119" s="1" t="s">
         <v>285</v>
-      </c>
-      <c r="C119" t="s">
-        <v>21</v>
-      </c>
-      <c r="D119" s="1" t="s">
-        <v>286</v>
       </c>
     </row>
     <row r="120" spans="1:7">
@@ -4886,13 +4973,13 @@
         <v>1002</v>
       </c>
       <c r="B120" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="C120" t="s">
         <v>287</v>
       </c>
-      <c r="C120" t="s">
+      <c r="D120" s="1" t="s">
         <v>288</v>
-      </c>
-      <c r="D120" s="1" t="s">
-        <v>289</v>
       </c>
     </row>
     <row r="121" spans="1:7">
@@ -4900,13 +4987,13 @@
         <v>1003</v>
       </c>
       <c r="B121" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="C121" t="s">
+        <v>287</v>
+      </c>
+      <c r="D121" s="1" t="s">
         <v>290</v>
-      </c>
-      <c r="C121" t="s">
-        <v>288</v>
-      </c>
-      <c r="D121" s="1" t="s">
-        <v>291</v>
       </c>
     </row>
     <row r="122" spans="1:7">
@@ -4914,13 +5001,13 @@
         <v>1024</v>
       </c>
       <c r="B122" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="C122" t="s">
+        <v>287</v>
+      </c>
+      <c r="D122" s="1" t="s">
         <v>292</v>
-      </c>
-      <c r="C122" t="s">
-        <v>288</v>
-      </c>
-      <c r="D122" s="1" t="s">
-        <v>293</v>
       </c>
     </row>
     <row r="123" spans="1:7">
@@ -4928,13 +5015,13 @@
         <v>1035</v>
       </c>
       <c r="B123" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="C123" t="s">
+        <v>287</v>
+      </c>
+      <c r="D123" s="1" t="s">
         <v>294</v>
-      </c>
-      <c r="C123" t="s">
-        <v>288</v>
-      </c>
-      <c r="D123" s="1" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="124" spans="1:7">
@@ -4942,13 +5029,13 @@
         <v>1037</v>
       </c>
       <c r="B124" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="C124" t="s">
+        <v>287</v>
+      </c>
+      <c r="D124" s="1" t="s">
         <v>296</v>
-      </c>
-      <c r="C124" t="s">
-        <v>288</v>
-      </c>
-      <c r="D124" s="1" t="s">
-        <v>297</v>
       </c>
     </row>
     <row r="125" ht="36" spans="1:7">
@@ -4956,13 +5043,13 @@
         <v>1038</v>
       </c>
       <c r="B125" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="C125" t="s">
+        <v>287</v>
+      </c>
+      <c r="D125" s="1" t="s">
         <v>298</v>
-      </c>
-      <c r="C125" t="s">
-        <v>288</v>
-      </c>
-      <c r="D125" s="1" t="s">
-        <v>299</v>
       </c>
     </row>
     <row r="126" spans="1:7">
@@ -4970,13 +5057,13 @@
         <v>1040</v>
       </c>
       <c r="B126" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="C126" t="s">
+        <v>287</v>
+      </c>
+      <c r="D126" s="1" t="s">
         <v>300</v>
-      </c>
-      <c r="C126" t="s">
-        <v>288</v>
-      </c>
-      <c r="D126" s="1" t="s">
-        <v>301</v>
       </c>
     </row>
     <row r="127" spans="1:7">
@@ -4984,13 +5071,13 @@
         <v>1041</v>
       </c>
       <c r="B127" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="C127" t="s">
+        <v>287</v>
+      </c>
+      <c r="D127" s="1" t="s">
         <v>302</v>
-      </c>
-      <c r="C127" t="s">
-        <v>288</v>
-      </c>
-      <c r="D127" s="1" t="s">
-        <v>303</v>
       </c>
     </row>
     <row r="128" spans="1:7">
@@ -4998,13 +5085,13 @@
         <v>1043</v>
       </c>
       <c r="B128" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="C128" t="s">
+        <v>287</v>
+      </c>
+      <c r="D128" s="1" t="s">
         <v>304</v>
-      </c>
-      <c r="C128" t="s">
-        <v>288</v>
-      </c>
-      <c r="D128" s="1" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="129" ht="36" spans="1:10">
@@ -5012,13 +5099,13 @@
         <v>1045</v>
       </c>
       <c r="B129" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="C129" t="s">
+        <v>287</v>
+      </c>
+      <c r="D129" s="1" t="s">
         <v>306</v>
-      </c>
-      <c r="C129" t="s">
-        <v>288</v>
-      </c>
-      <c r="D129" s="1" t="s">
-        <v>307</v>
       </c>
     </row>
     <row r="130" spans="1:10">
@@ -5026,13 +5113,13 @@
         <v>1053</v>
       </c>
       <c r="B130" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="C130" t="s">
+        <v>287</v>
+      </c>
+      <c r="D130" s="1" t="s">
         <v>308</v>
-      </c>
-      <c r="C130" t="s">
-        <v>288</v>
-      </c>
-      <c r="D130" s="1" t="s">
-        <v>309</v>
       </c>
     </row>
     <row r="131" spans="1:10">
@@ -5040,13 +5127,13 @@
         <v>1059</v>
       </c>
       <c r="B131" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="C131" t="s">
+        <v>287</v>
+      </c>
+      <c r="D131" s="1" t="s">
         <v>310</v>
-      </c>
-      <c r="C131" t="s">
-        <v>288</v>
-      </c>
-      <c r="D131" s="1" t="s">
-        <v>311</v>
       </c>
     </row>
     <row r="132" spans="1:10">
@@ -5054,13 +5141,13 @@
         <v>1060</v>
       </c>
       <c r="B132" s="1" t="s">
+        <v>311</v>
+      </c>
+      <c r="C132" t="s">
+        <v>287</v>
+      </c>
+      <c r="D132" s="1" t="s">
         <v>312</v>
-      </c>
-      <c r="C132" t="s">
-        <v>288</v>
-      </c>
-      <c r="D132" s="1" t="s">
-        <v>313</v>
       </c>
       <c r="F132" t="s">
         <v>14</v>
@@ -5069,7 +5156,7 @@
         <v>16</v>
       </c>
       <c r="I132" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="133" spans="1:10">
@@ -5077,13 +5164,13 @@
         <v>1061</v>
       </c>
       <c r="B133" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="C133" t="s">
+        <v>287</v>
+      </c>
+      <c r="D133" s="1" t="s">
         <v>315</v>
-      </c>
-      <c r="C133" t="s">
-        <v>288</v>
-      </c>
-      <c r="D133" s="1" t="s">
-        <v>316</v>
       </c>
       <c r="F133" t="s">
         <v>14</v>
@@ -5092,7 +5179,7 @@
         <v>16</v>
       </c>
       <c r="I133" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="134" spans="1:10">
@@ -5100,13 +5187,13 @@
         <v>1063</v>
       </c>
       <c r="B134" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="C134" t="s">
+        <v>287</v>
+      </c>
+      <c r="D134" s="1" t="s">
         <v>318</v>
-      </c>
-      <c r="C134" t="s">
-        <v>288</v>
-      </c>
-      <c r="D134" s="1" t="s">
-        <v>319</v>
       </c>
     </row>
     <row r="135" spans="1:10">
@@ -5114,13 +5201,13 @@
         <v>1064</v>
       </c>
       <c r="B135" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="C135" t="s">
+        <v>287</v>
+      </c>
+      <c r="D135" s="1" t="s">
         <v>320</v>
-      </c>
-      <c r="C135" t="s">
-        <v>288</v>
-      </c>
-      <c r="D135" s="1" t="s">
-        <v>321</v>
       </c>
     </row>
     <row r="136" spans="1:10">
@@ -5128,13 +5215,13 @@
         <v>1069</v>
       </c>
       <c r="B136" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="C136" t="s">
+        <v>287</v>
+      </c>
+      <c r="D136" s="1" t="s">
         <v>322</v>
-      </c>
-      <c r="C136" t="s">
-        <v>288</v>
-      </c>
-      <c r="D136" s="1" t="s">
-        <v>323</v>
       </c>
     </row>
     <row r="137" spans="1:10">
@@ -5142,13 +5229,13 @@
         <v>1077</v>
       </c>
       <c r="B137" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="C137" t="s">
+        <v>287</v>
+      </c>
+      <c r="D137" s="1" t="s">
         <v>324</v>
-      </c>
-      <c r="C137" t="s">
-        <v>288</v>
-      </c>
-      <c r="D137" s="1" t="s">
-        <v>325</v>
       </c>
     </row>
     <row r="138" spans="1:10">
@@ -5156,13 +5243,13 @@
         <v>1088</v>
       </c>
       <c r="B138" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="C138" t="s">
+        <v>287</v>
+      </c>
+      <c r="D138" s="1" t="s">
         <v>326</v>
-      </c>
-      <c r="C138" t="s">
-        <v>288</v>
-      </c>
-      <c r="D138" s="1" t="s">
-        <v>327</v>
       </c>
     </row>
     <row r="139" spans="1:10">
@@ -5170,13 +5257,13 @@
         <v>2000</v>
       </c>
       <c r="B139" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="C139" t="s">
+        <v>11</v>
+      </c>
+      <c r="D139" s="1" t="s">
         <v>328</v>
-      </c>
-      <c r="C139" t="s">
-        <v>11</v>
-      </c>
-      <c r="D139" s="1" t="s">
-        <v>329</v>
       </c>
       <c r="E139" t="s">
         <v>13</v>
@@ -5188,10 +5275,10 @@
         <v>15</v>
       </c>
       <c r="H139" t="s">
+        <v>329</v>
+      </c>
+      <c r="I139" t="s">
         <v>330</v>
-      </c>
-      <c r="I139" t="s">
-        <v>331</v>
       </c>
     </row>
     <row r="140" spans="1:10">
@@ -5199,13 +5286,13 @@
         <v>2001</v>
       </c>
       <c r="B140" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="C140" t="s">
+        <v>21</v>
+      </c>
+      <c r="D140" s="1" t="s">
         <v>332</v>
-      </c>
-      <c r="C140" t="s">
-        <v>21</v>
-      </c>
-      <c r="D140" s="1" t="s">
-        <v>333</v>
       </c>
       <c r="E140" t="s">
         <v>13</v>
@@ -5217,13 +5304,13 @@
         <v>201</v>
       </c>
       <c r="H140" t="s">
+        <v>333</v>
+      </c>
+      <c r="I140" t="s">
         <v>334</v>
       </c>
-      <c r="I140" t="s">
+      <c r="J140" t="s">
         <v>335</v>
-      </c>
-      <c r="J140" t="s">
-        <v>336</v>
       </c>
     </row>
     <row r="141" spans="1:10">
@@ -5231,31 +5318,31 @@
         <v>2002</v>
       </c>
       <c r="B141" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="C141" t="s">
+        <v>21</v>
+      </c>
+      <c r="D141" s="1" t="s">
         <v>337</v>
       </c>
-      <c r="C141" t="s">
-        <v>21</v>
-      </c>
-      <c r="D141" s="1" t="s">
+      <c r="E141" t="s">
+        <v>13</v>
+      </c>
+      <c r="F141" t="s">
+        <v>13</v>
+      </c>
+      <c r="G141" t="s">
         <v>338</v>
       </c>
-      <c r="E141" t="s">
-        <v>13</v>
-      </c>
-      <c r="F141" t="s">
-        <v>13</v>
-      </c>
-      <c r="G141" t="s">
+      <c r="H141" t="s">
         <v>339</v>
       </c>
-      <c r="H141" t="s">
+      <c r="I141" t="s">
         <v>340</v>
       </c>
-      <c r="I141" t="s">
+      <c r="J141" t="s">
         <v>341</v>
-      </c>
-      <c r="J141" t="s">
-        <v>342</v>
       </c>
     </row>
     <row r="142" spans="1:10">
@@ -5263,13 +5350,13 @@
         <v>2003</v>
       </c>
       <c r="B142" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="C142" t="s">
+        <v>11</v>
+      </c>
+      <c r="D142" s="1" t="s">
         <v>343</v>
-      </c>
-      <c r="C142" t="s">
-        <v>11</v>
-      </c>
-      <c r="D142" s="1" t="s">
-        <v>344</v>
       </c>
       <c r="E142" t="s">
         <v>13</v>
@@ -5281,10 +5368,10 @@
         <v>15</v>
       </c>
       <c r="H142" t="s">
+        <v>344</v>
+      </c>
+      <c r="I142" t="s">
         <v>345</v>
-      </c>
-      <c r="I142" t="s">
-        <v>346</v>
       </c>
     </row>
     <row r="143" spans="1:10">
@@ -5292,31 +5379,31 @@
         <v>2004</v>
       </c>
       <c r="B143" s="1" t="s">
+        <v>346</v>
+      </c>
+      <c r="C143" t="s">
+        <v>21</v>
+      </c>
+      <c r="D143" s="1" t="s">
         <v>347</v>
       </c>
-      <c r="C143" t="s">
-        <v>21</v>
-      </c>
-      <c r="D143" s="1" t="s">
+      <c r="E143" t="s">
+        <v>13</v>
+      </c>
+      <c r="F143" t="s">
+        <v>13</v>
+      </c>
+      <c r="G143" t="s">
         <v>348</v>
       </c>
-      <c r="E143" t="s">
-        <v>13</v>
-      </c>
-      <c r="F143" t="s">
-        <v>13</v>
-      </c>
-      <c r="G143" t="s">
+      <c r="H143" t="s">
         <v>349</v>
       </c>
-      <c r="H143" t="s">
+      <c r="I143" t="s">
         <v>350</v>
       </c>
-      <c r="I143" t="s">
+      <c r="J143" t="s">
         <v>351</v>
-      </c>
-      <c r="J143" t="s">
-        <v>352</v>
       </c>
     </row>
     <row r="144" spans="1:10">
@@ -5324,19 +5411,22 @@
         <v>2005</v>
       </c>
       <c r="B144" s="1" t="s">
+        <v>352</v>
+      </c>
+      <c r="C144" t="s">
+        <v>21</v>
+      </c>
+      <c r="D144" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="C144" t="s">
-        <v>21</v>
-      </c>
-      <c r="D144" s="1" t="s">
+      <c r="E144" t="s">
+        <v>13</v>
+      </c>
+      <c r="F144" t="s">
+        <v>32</v>
+      </c>
+      <c r="G144" t="s">
         <v>354</v>
-      </c>
-      <c r="E144" t="s">
-        <v>13</v>
-      </c>
-      <c r="G144" t="s">
-        <v>355</v>
       </c>
     </row>
     <row r="145" spans="1:10">
@@ -5344,19 +5434,22 @@
         <v>2006</v>
       </c>
       <c r="B145" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="C145" t="s">
+        <v>21</v>
+      </c>
+      <c r="D145" s="1" t="s">
         <v>356</v>
       </c>
-      <c r="C145" t="s">
-        <v>21</v>
-      </c>
-      <c r="D145" s="1" t="s">
+      <c r="E145" t="s">
+        <v>13</v>
+      </c>
+      <c r="F145" t="s">
+        <v>32</v>
+      </c>
+      <c r="G145" t="s">
         <v>357</v>
-      </c>
-      <c r="E145" t="s">
-        <v>13</v>
-      </c>
-      <c r="G145" t="s">
-        <v>358</v>
       </c>
     </row>
     <row r="146" spans="1:10">
@@ -5364,13 +5457,13 @@
         <v>2007</v>
       </c>
       <c r="B146" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="C146" t="s">
+        <v>21</v>
+      </c>
+      <c r="D146" s="1" t="s">
         <v>359</v>
-      </c>
-      <c r="C146" t="s">
-        <v>21</v>
-      </c>
-      <c r="D146" s="1" t="s">
-        <v>360</v>
       </c>
     </row>
     <row r="147" spans="1:10">
@@ -5378,19 +5471,22 @@
         <v>2008</v>
       </c>
       <c r="B147" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="C147" t="s">
+        <v>21</v>
+      </c>
+      <c r="D147" s="1" t="s">
         <v>361</v>
       </c>
-      <c r="C147" t="s">
-        <v>21</v>
-      </c>
-      <c r="D147" s="1" t="s">
-        <v>362</v>
-      </c>
       <c r="E147" t="s">
         <v>13</v>
       </c>
+      <c r="F147" t="s">
+        <v>32</v>
+      </c>
       <c r="G147" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="148" spans="1:10">
@@ -5398,19 +5494,22 @@
         <v>2009</v>
       </c>
       <c r="B148" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="C148" t="s">
+        <v>21</v>
+      </c>
+      <c r="D148" s="1" t="s">
         <v>363</v>
       </c>
-      <c r="C148" t="s">
-        <v>21</v>
-      </c>
-      <c r="D148" s="1" t="s">
-        <v>364</v>
-      </c>
       <c r="E148" t="s">
         <v>13</v>
       </c>
+      <c r="F148" t="s">
+        <v>32</v>
+      </c>
       <c r="G148" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="149" spans="1:10">
@@ -5418,19 +5517,22 @@
         <v>2010</v>
       </c>
       <c r="B149" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="C149" t="s">
+        <v>21</v>
+      </c>
+      <c r="D149" s="1" t="s">
         <v>365</v>
       </c>
-      <c r="C149" t="s">
-        <v>21</v>
-      </c>
-      <c r="D149" s="1" t="s">
+      <c r="E149" t="s">
+        <v>13</v>
+      </c>
+      <c r="F149" t="s">
+        <v>32</v>
+      </c>
+      <c r="G149" t="s">
         <v>366</v>
-      </c>
-      <c r="E149" t="s">
-        <v>13</v>
-      </c>
-      <c r="G149" t="s">
-        <v>367</v>
       </c>
     </row>
     <row r="150" spans="1:10">
@@ -5438,13 +5540,13 @@
         <v>2011</v>
       </c>
       <c r="B150" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="C150" t="s">
+        <v>21</v>
+      </c>
+      <c r="D150" s="1" t="s">
         <v>368</v>
-      </c>
-      <c r="C150" t="s">
-        <v>21</v>
-      </c>
-      <c r="D150" s="1" t="s">
-        <v>369</v>
       </c>
     </row>
     <row r="151" spans="1:10">
@@ -5452,16 +5554,19 @@
         <v>2012</v>
       </c>
       <c r="B151" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="C151" t="s">
+        <v>21</v>
+      </c>
+      <c r="D151" s="1" t="s">
         <v>370</v>
       </c>
-      <c r="C151" t="s">
-        <v>21</v>
-      </c>
-      <c r="D151" s="1" t="s">
-        <v>371</v>
-      </c>
       <c r="E151" t="s">
         <v>13</v>
+      </c>
+      <c r="F151" t="s">
+        <v>32</v>
       </c>
       <c r="G151" t="s">
         <v>122</v>
@@ -5472,16 +5577,19 @@
         <v>2013</v>
       </c>
       <c r="B152" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="C152" t="s">
+        <v>21</v>
+      </c>
+      <c r="D152" s="1" t="s">
         <v>372</v>
       </c>
-      <c r="C152" t="s">
-        <v>21</v>
-      </c>
-      <c r="D152" s="1" t="s">
-        <v>373</v>
-      </c>
       <c r="E152" t="s">
         <v>13</v>
+      </c>
+      <c r="F152" t="s">
+        <v>32</v>
       </c>
       <c r="G152" t="s">
         <v>119</v>
@@ -5492,19 +5600,22 @@
         <v>2014</v>
       </c>
       <c r="B153" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="C153" t="s">
+        <v>21</v>
+      </c>
+      <c r="D153" s="1" t="s">
         <v>374</v>
       </c>
-      <c r="C153" t="s">
-        <v>21</v>
-      </c>
-      <c r="D153" s="1" t="s">
+      <c r="E153" t="s">
+        <v>13</v>
+      </c>
+      <c r="F153" t="s">
+        <v>32</v>
+      </c>
+      <c r="G153" t="s">
         <v>375</v>
-      </c>
-      <c r="E153" t="s">
-        <v>13</v>
-      </c>
-      <c r="G153" t="s">
-        <v>376</v>
       </c>
     </row>
     <row r="154" spans="1:10">
@@ -5512,19 +5623,22 @@
         <v>2015</v>
       </c>
       <c r="B154" s="1" t="s">
+        <v>376</v>
+      </c>
+      <c r="C154" t="s">
+        <v>21</v>
+      </c>
+      <c r="D154" s="1" t="s">
         <v>377</v>
       </c>
-      <c r="C154" t="s">
-        <v>21</v>
-      </c>
-      <c r="D154" s="1" t="s">
+      <c r="E154" t="s">
+        <v>13</v>
+      </c>
+      <c r="F154" t="s">
+        <v>32</v>
+      </c>
+      <c r="G154" t="s">
         <v>378</v>
-      </c>
-      <c r="E154" t="s">
-        <v>13</v>
-      </c>
-      <c r="G154" t="s">
-        <v>379</v>
       </c>
     </row>
     <row r="155" ht="36" spans="1:10">
@@ -5532,13 +5646,13 @@
         <v>2016</v>
       </c>
       <c r="B155" s="1" t="s">
+        <v>379</v>
+      </c>
+      <c r="C155" t="s">
+        <v>11</v>
+      </c>
+      <c r="D155" s="1" t="s">
         <v>380</v>
-      </c>
-      <c r="C155" t="s">
-        <v>11</v>
-      </c>
-      <c r="D155" s="1" t="s">
-        <v>381</v>
       </c>
       <c r="E155" t="s">
         <v>13</v>
@@ -5550,10 +5664,10 @@
         <v>15</v>
       </c>
       <c r="H155" t="s">
+        <v>381</v>
+      </c>
+      <c r="I155" t="s">
         <v>382</v>
-      </c>
-      <c r="I155" t="s">
-        <v>383</v>
       </c>
     </row>
     <row r="156" ht="36" spans="1:10">
@@ -5561,13 +5675,13 @@
         <v>2017</v>
       </c>
       <c r="B156" s="1" t="s">
+        <v>383</v>
+      </c>
+      <c r="C156" t="s">
+        <v>21</v>
+      </c>
+      <c r="D156" s="1" t="s">
         <v>384</v>
-      </c>
-      <c r="C156" t="s">
-        <v>21</v>
-      </c>
-      <c r="D156" s="1" t="s">
-        <v>385</v>
       </c>
       <c r="E156" t="s">
         <v>13</v>
@@ -5579,13 +5693,13 @@
         <v>204</v>
       </c>
       <c r="H156" t="s">
+        <v>385</v>
+      </c>
+      <c r="I156" t="s">
         <v>386</v>
       </c>
-      <c r="I156" t="s">
+      <c r="J156" t="s">
         <v>387</v>
-      </c>
-      <c r="J156" t="s">
-        <v>388</v>
       </c>
     </row>
     <row r="157" ht="36" spans="1:10">
@@ -5593,31 +5707,31 @@
         <v>2018</v>
       </c>
       <c r="B157" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="C157" t="s">
+        <v>21</v>
+      </c>
+      <c r="D157" s="1" t="s">
         <v>389</v>
       </c>
-      <c r="C157" t="s">
-        <v>21</v>
-      </c>
-      <c r="D157" s="1" t="s">
+      <c r="E157" t="s">
+        <v>13</v>
+      </c>
+      <c r="F157" t="s">
+        <v>13</v>
+      </c>
+      <c r="G157" t="s">
         <v>390</v>
       </c>
-      <c r="E157" t="s">
-        <v>13</v>
-      </c>
-      <c r="F157" t="s">
-        <v>13</v>
-      </c>
-      <c r="G157" t="s">
+      <c r="H157" t="s">
         <v>391</v>
       </c>
-      <c r="H157" t="s">
+      <c r="I157" t="s">
         <v>392</v>
       </c>
-      <c r="I157" t="s">
+      <c r="J157" t="s">
         <v>393</v>
-      </c>
-      <c r="J157" t="s">
-        <v>394</v>
       </c>
     </row>
     <row r="158" ht="36" spans="1:10">
@@ -5625,13 +5739,13 @@
         <v>2025</v>
       </c>
       <c r="B158" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="C158" t="s">
+        <v>11</v>
+      </c>
+      <c r="D158" s="1" t="s">
         <v>395</v>
-      </c>
-      <c r="C158" t="s">
-        <v>11</v>
-      </c>
-      <c r="D158" s="1" t="s">
-        <v>396</v>
       </c>
       <c r="E158" t="s">
         <v>13</v>
@@ -5643,10 +5757,10 @@
         <v>15</v>
       </c>
       <c r="H158" t="s">
+        <v>396</v>
+      </c>
+      <c r="I158" t="s">
         <v>397</v>
-      </c>
-      <c r="I158" t="s">
-        <v>398</v>
       </c>
     </row>
     <row r="159" ht="36" spans="1:10">
@@ -5654,13 +5768,13 @@
         <v>2026</v>
       </c>
       <c r="B159" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="C159" t="s">
+        <v>21</v>
+      </c>
+      <c r="D159" s="1" t="s">
         <v>399</v>
-      </c>
-      <c r="C159" t="s">
-        <v>21</v>
-      </c>
-      <c r="D159" s="1" t="s">
-        <v>400</v>
       </c>
       <c r="E159" t="s">
         <v>13</v>
@@ -5672,13 +5786,13 @@
         <v>204</v>
       </c>
       <c r="H159" t="s">
+        <v>400</v>
+      </c>
+      <c r="I159" t="s">
         <v>401</v>
       </c>
-      <c r="I159" t="s">
+      <c r="J159" t="s">
         <v>402</v>
-      </c>
-      <c r="J159" t="s">
-        <v>403</v>
       </c>
     </row>
     <row r="160" ht="36" spans="1:10">
@@ -5686,31 +5800,31 @@
         <v>2027</v>
       </c>
       <c r="B160" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="C160" t="s">
+        <v>21</v>
+      </c>
+      <c r="D160" s="1" t="s">
         <v>404</v>
       </c>
-      <c r="C160" t="s">
-        <v>21</v>
-      </c>
-      <c r="D160" s="1" t="s">
+      <c r="E160" t="s">
+        <v>13</v>
+      </c>
+      <c r="F160" t="s">
+        <v>13</v>
+      </c>
+      <c r="G160" t="s">
+        <v>390</v>
+      </c>
+      <c r="H160" t="s">
         <v>405</v>
       </c>
-      <c r="E160" t="s">
-        <v>13</v>
-      </c>
-      <c r="F160" t="s">
-        <v>13</v>
-      </c>
-      <c r="G160" t="s">
-        <v>391</v>
-      </c>
-      <c r="H160" t="s">
+      <c r="I160" t="s">
         <v>406</v>
       </c>
-      <c r="I160" t="s">
+      <c r="J160" t="s">
         <v>407</v>
-      </c>
-      <c r="J160" t="s">
-        <v>408</v>
       </c>
     </row>
     <row r="161" ht="54" spans="1:7">
@@ -5718,13 +5832,13 @@
         <v>2028</v>
       </c>
       <c r="B161" s="1" t="s">
+        <v>408</v>
+      </c>
+      <c r="C161" t="s">
+        <v>21</v>
+      </c>
+      <c r="D161" s="1" t="s">
         <v>409</v>
-      </c>
-      <c r="C161" t="s">
-        <v>21</v>
-      </c>
-      <c r="D161" s="1" t="s">
-        <v>410</v>
       </c>
     </row>
     <row r="162" ht="54" spans="1:7">
@@ -5732,13 +5846,13 @@
         <v>2029</v>
       </c>
       <c r="B162" s="1" t="s">
+        <v>410</v>
+      </c>
+      <c r="C162" t="s">
+        <v>11</v>
+      </c>
+      <c r="D162" s="1" t="s">
         <v>411</v>
-      </c>
-      <c r="C162" t="s">
-        <v>11</v>
-      </c>
-      <c r="D162" s="1" t="s">
-        <v>412</v>
       </c>
     </row>
     <row r="163" spans="1:7">
@@ -5746,13 +5860,13 @@
         <v>2030</v>
       </c>
       <c r="B163" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="C163" t="s">
+        <v>21</v>
+      </c>
+      <c r="D163" s="1" t="s">
         <v>413</v>
-      </c>
-      <c r="C163" t="s">
-        <v>21</v>
-      </c>
-      <c r="D163" s="1" t="s">
-        <v>414</v>
       </c>
     </row>
     <row r="164" spans="1:7">
@@ -5760,13 +5874,13 @@
         <v>2031</v>
       </c>
       <c r="B164" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="C164" t="s">
+        <v>21</v>
+      </c>
+      <c r="D164" s="1" t="s">
         <v>415</v>
-      </c>
-      <c r="C164" t="s">
-        <v>21</v>
-      </c>
-      <c r="D164" s="1" t="s">
-        <v>416</v>
       </c>
     </row>
     <row r="165" ht="36" spans="1:7">
@@ -5774,13 +5888,13 @@
         <v>2032</v>
       </c>
       <c r="B165" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="C165" t="s">
+        <v>11</v>
+      </c>
+      <c r="D165" s="1" t="s">
         <v>417</v>
-      </c>
-      <c r="C165" t="s">
-        <v>11</v>
-      </c>
-      <c r="D165" s="1" t="s">
-        <v>418</v>
       </c>
     </row>
     <row r="166" spans="1:7">
@@ -5788,13 +5902,13 @@
         <v>2034</v>
       </c>
       <c r="B166" s="1" t="s">
+        <v>418</v>
+      </c>
+      <c r="C166" t="s">
+        <v>11</v>
+      </c>
+      <c r="D166" s="1" t="s">
         <v>419</v>
-      </c>
-      <c r="C166" t="s">
-        <v>11</v>
-      </c>
-      <c r="D166" s="1" t="s">
-        <v>420</v>
       </c>
     </row>
     <row r="167" spans="1:7">
@@ -5802,13 +5916,13 @@
         <v>2035</v>
       </c>
       <c r="B167" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="C167" t="s">
+        <v>11</v>
+      </c>
+      <c r="D167" s="1" t="s">
         <v>421</v>
-      </c>
-      <c r="C167" t="s">
-        <v>11</v>
-      </c>
-      <c r="D167" s="1" t="s">
-        <v>422</v>
       </c>
     </row>
     <row r="168" ht="54" spans="1:7">
@@ -5816,13 +5930,13 @@
         <v>2036</v>
       </c>
       <c r="B168" s="1" t="s">
+        <v>422</v>
+      </c>
+      <c r="C168" t="s">
+        <v>11</v>
+      </c>
+      <c r="D168" s="1" t="s">
         <v>423</v>
-      </c>
-      <c r="C168" t="s">
-        <v>11</v>
-      </c>
-      <c r="D168" s="1" t="s">
-        <v>424</v>
       </c>
     </row>
     <row r="169" spans="1:7">
@@ -5830,13 +5944,13 @@
         <v>2037</v>
       </c>
       <c r="B169" s="1" t="s">
+        <v>424</v>
+      </c>
+      <c r="C169" t="s">
+        <v>11</v>
+      </c>
+      <c r="D169" s="1" t="s">
         <v>425</v>
-      </c>
-      <c r="C169" t="s">
-        <v>11</v>
-      </c>
-      <c r="D169" s="1" t="s">
-        <v>426</v>
       </c>
     </row>
     <row r="170" spans="1:7">
@@ -5844,13 +5958,13 @@
         <v>2038</v>
       </c>
       <c r="B170" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="C170" t="s">
+        <v>21</v>
+      </c>
+      <c r="D170" s="1" t="s">
         <v>427</v>
-      </c>
-      <c r="C170" t="s">
-        <v>21</v>
-      </c>
-      <c r="D170" s="1" t="s">
-        <v>428</v>
       </c>
     </row>
     <row r="171" spans="1:7">
@@ -5858,13 +5972,13 @@
         <v>2040</v>
       </c>
       <c r="B171" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="C171" t="s">
+        <v>11</v>
+      </c>
+      <c r="D171" s="1" t="s">
         <v>429</v>
-      </c>
-      <c r="C171" t="s">
-        <v>11</v>
-      </c>
-      <c r="D171" s="1" t="s">
-        <v>430</v>
       </c>
     </row>
     <row r="172" spans="1:7">
@@ -5872,16 +5986,19 @@
         <v>2052</v>
       </c>
       <c r="B172" s="1" t="s">
+        <v>430</v>
+      </c>
+      <c r="C172" t="s">
+        <v>21</v>
+      </c>
+      <c r="D172" s="1" t="s">
         <v>431</v>
       </c>
-      <c r="C172" t="s">
-        <v>21</v>
-      </c>
-      <c r="D172" s="1" t="s">
-        <v>432</v>
-      </c>
       <c r="E172" t="s">
         <v>13</v>
+      </c>
+      <c r="F172" t="s">
+        <v>32</v>
       </c>
       <c r="G172" t="s">
         <v>122</v>
@@ -5892,16 +6009,19 @@
         <v>3004</v>
       </c>
       <c r="B173" s="1" t="s">
+        <v>432</v>
+      </c>
+      <c r="C173" t="s">
+        <v>11</v>
+      </c>
+      <c r="D173" s="1" t="s">
         <v>433</v>
       </c>
-      <c r="C173" t="s">
-        <v>11</v>
-      </c>
-      <c r="D173" s="1" t="s">
-        <v>434</v>
-      </c>
       <c r="E173" t="s">
         <v>13</v>
+      </c>
+      <c r="F173" t="s">
+        <v>32</v>
       </c>
       <c r="G173" t="s">
         <v>15</v>
@@ -5912,13 +6032,13 @@
         <v>3007</v>
       </c>
       <c r="B174" s="1" t="s">
+        <v>434</v>
+      </c>
+      <c r="C174" t="s">
+        <v>11</v>
+      </c>
+      <c r="D174" s="1" t="s">
         <v>435</v>
-      </c>
-      <c r="C174" t="s">
-        <v>11</v>
-      </c>
-      <c r="D174" s="1" t="s">
-        <v>436</v>
       </c>
     </row>
     <row r="175" ht="36" spans="1:7">
@@ -5926,13 +6046,13 @@
         <v>3008</v>
       </c>
       <c r="B175" s="1" t="s">
+        <v>436</v>
+      </c>
+      <c r="C175" t="s">
+        <v>11</v>
+      </c>
+      <c r="D175" s="1" t="s">
         <v>437</v>
-      </c>
-      <c r="C175" t="s">
-        <v>11</v>
-      </c>
-      <c r="D175" s="1" t="s">
-        <v>438</v>
       </c>
     </row>
     <row r="176" spans="1:7">
@@ -5940,16 +6060,19 @@
         <v>3009</v>
       </c>
       <c r="B176" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="C176" t="s">
+        <v>11</v>
+      </c>
+      <c r="D176" s="1" t="s">
         <v>439</v>
       </c>
-      <c r="C176" t="s">
-        <v>11</v>
-      </c>
-      <c r="D176" s="1" t="s">
-        <v>440</v>
-      </c>
       <c r="E176" t="s">
         <v>13</v>
+      </c>
+      <c r="F176" t="s">
+        <v>32</v>
       </c>
       <c r="G176" t="s">
         <v>15</v>
@@ -5960,16 +6083,19 @@
         <v>3010</v>
       </c>
       <c r="B177" s="1" t="s">
+        <v>440</v>
+      </c>
+      <c r="C177" t="s">
+        <v>11</v>
+      </c>
+      <c r="D177" s="1" t="s">
         <v>441</v>
       </c>
-      <c r="C177" t="s">
-        <v>11</v>
-      </c>
-      <c r="D177" s="1" t="s">
-        <v>442</v>
-      </c>
       <c r="E177" t="s">
         <v>13</v>
+      </c>
+      <c r="F177" t="s">
+        <v>32</v>
       </c>
       <c r="G177" t="s">
         <v>15</v>
@@ -5980,13 +6106,13 @@
         <v>3011</v>
       </c>
       <c r="B178" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="C178" t="s">
+        <v>11</v>
+      </c>
+      <c r="D178" s="1" t="s">
         <v>443</v>
-      </c>
-      <c r="C178" t="s">
-        <v>11</v>
-      </c>
-      <c r="D178" s="1" t="s">
-        <v>444</v>
       </c>
     </row>
     <row r="179" ht="54" spans="1:7">
@@ -5994,13 +6120,13 @@
         <v>3012</v>
       </c>
       <c r="B179" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="C179" t="s">
+        <v>11</v>
+      </c>
+      <c r="D179" s="1" t="s">
         <v>445</v>
-      </c>
-      <c r="C179" t="s">
-        <v>11</v>
-      </c>
-      <c r="D179" s="1" t="s">
-        <v>446</v>
       </c>
     </row>
     <row r="180" ht="36" spans="1:7">
@@ -6008,13 +6134,13 @@
         <v>3024</v>
       </c>
       <c r="B180" s="1" t="s">
+        <v>446</v>
+      </c>
+      <c r="C180" t="s">
+        <v>21</v>
+      </c>
+      <c r="D180" s="1" t="s">
         <v>447</v>
-      </c>
-      <c r="C180" t="s">
-        <v>21</v>
-      </c>
-      <c r="D180" s="1" t="s">
-        <v>448</v>
       </c>
     </row>
     <row r="181" ht="54" spans="1:7">
@@ -6022,13 +6148,13 @@
         <v>3027</v>
       </c>
       <c r="B181" s="1" t="s">
+        <v>448</v>
+      </c>
+      <c r="C181" t="s">
+        <v>21</v>
+      </c>
+      <c r="D181" s="1" t="s">
         <v>449</v>
-      </c>
-      <c r="C181" t="s">
-        <v>21</v>
-      </c>
-      <c r="D181" s="1" t="s">
-        <v>450</v>
       </c>
     </row>
     <row r="182" ht="54" spans="1:7">
@@ -6036,13 +6162,13 @@
         <v>3028</v>
       </c>
       <c r="B182" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="C182" t="s">
+        <v>21</v>
+      </c>
+      <c r="D182" s="1" t="s">
         <v>451</v>
-      </c>
-      <c r="C182" t="s">
-        <v>21</v>
-      </c>
-      <c r="D182" s="1" t="s">
-        <v>452</v>
       </c>
     </row>
     <row r="183" ht="36" spans="1:7">
@@ -6050,13 +6176,13 @@
         <v>4029</v>
       </c>
       <c r="B183" s="1" t="s">
+        <v>452</v>
+      </c>
+      <c r="C183" t="s">
+        <v>287</v>
+      </c>
+      <c r="D183" s="1" t="s">
         <v>453</v>
-      </c>
-      <c r="C183" t="s">
-        <v>288</v>
-      </c>
-      <c r="D183" s="1" t="s">
-        <v>454</v>
       </c>
     </row>
     <row r="184" spans="1:7">
@@ -6064,13 +6190,13 @@
         <v>5013</v>
       </c>
       <c r="B184" s="1" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="C184" t="s">
         <v>24</v>
       </c>
       <c r="D184" s="1" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="185" ht="36" spans="1:7">
@@ -6078,19 +6204,22 @@
         <v>5525</v>
       </c>
       <c r="B185" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="C185" t="s">
+        <v>21</v>
+      </c>
+      <c r="D185" s="1" t="s">
         <v>457</v>
       </c>
-      <c r="C185" t="s">
-        <v>21</v>
-      </c>
-      <c r="D185" s="1" t="s">
+      <c r="E185" t="s">
+        <v>13</v>
+      </c>
+      <c r="F185" t="s">
+        <v>32</v>
+      </c>
+      <c r="G185" t="s">
         <v>458</v>
-      </c>
-      <c r="E185" t="s">
-        <v>13</v>
-      </c>
-      <c r="G185" t="s">
-        <v>459</v>
       </c>
     </row>
     <row r="186" ht="90" spans="1:7">
@@ -6098,10 +6227,10 @@
         <v>5555</v>
       </c>
       <c r="B186" s="1" t="s">
+        <v>459</v>
+      </c>
+      <c r="D186" s="1" t="s">
         <v>460</v>
-      </c>
-      <c r="D186" s="1" t="s">
-        <v>461</v>
       </c>
     </row>
     <row r="187" spans="1:7">
@@ -6109,13 +6238,13 @@
         <v>8001</v>
       </c>
       <c r="B187" s="1" t="s">
+        <v>461</v>
+      </c>
+      <c r="C187" t="s">
+        <v>21</v>
+      </c>
+      <c r="D187" s="1" t="s">
         <v>462</v>
-      </c>
-      <c r="C187" t="s">
-        <v>21</v>
-      </c>
-      <c r="D187" s="1" t="s">
-        <v>463</v>
       </c>
     </row>
     <row r="188" spans="1:7">
@@ -6123,13 +6252,13 @@
         <v>8002</v>
       </c>
       <c r="B188" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="C188" t="s">
+        <v>287</v>
+      </c>
+      <c r="D188" s="1" t="s">
         <v>464</v>
-      </c>
-      <c r="C188" t="s">
-        <v>288</v>
-      </c>
-      <c r="D188" s="1" t="s">
-        <v>465</v>
       </c>
     </row>
     <row r="189" spans="1:7">
@@ -6137,13 +6266,13 @@
         <v>8003</v>
       </c>
       <c r="B189" s="1" t="s">
+        <v>465</v>
+      </c>
+      <c r="C189" t="s">
+        <v>287</v>
+      </c>
+      <c r="D189" s="1" t="s">
         <v>466</v>
-      </c>
-      <c r="C189" t="s">
-        <v>288</v>
-      </c>
-      <c r="D189" s="1" t="s">
-        <v>467</v>
       </c>
     </row>
     <row r="190" spans="1:7">
@@ -6151,13 +6280,13 @@
         <v>8004</v>
       </c>
       <c r="B190" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="C190" t="s">
+        <v>21</v>
+      </c>
+      <c r="D190" s="1" t="s">
         <v>468</v>
-      </c>
-      <c r="C190" t="s">
-        <v>21</v>
-      </c>
-      <c r="D190" s="1" t="s">
-        <v>469</v>
       </c>
     </row>
     <row r="191" spans="1:7">
@@ -6165,13 +6294,13 @@
         <v>8005</v>
       </c>
       <c r="B191" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="C191" t="s">
+        <v>21</v>
+      </c>
+      <c r="D191" s="1" t="s">
         <v>470</v>
-      </c>
-      <c r="C191" t="s">
-        <v>21</v>
-      </c>
-      <c r="D191" s="1" t="s">
-        <v>471</v>
       </c>
     </row>
     <row r="192" spans="1:7">
@@ -6179,13 +6308,13 @@
         <v>8006</v>
       </c>
       <c r="B192" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="C192" t="s">
+        <v>21</v>
+      </c>
+      <c r="D192" s="1" t="s">
         <v>472</v>
-      </c>
-      <c r="C192" t="s">
-        <v>21</v>
-      </c>
-      <c r="D192" s="1" t="s">
-        <v>473</v>
       </c>
     </row>
     <row r="193" spans="1:4">
@@ -6193,13 +6322,13 @@
         <v>8007</v>
       </c>
       <c r="B193" s="1" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="C193" t="s">
         <v>24</v>
       </c>
       <c r="D193" s="1" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="194" spans="1:4">
@@ -6207,13 +6336,13 @@
         <v>8008</v>
       </c>
       <c r="B194" s="1" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="C194" t="s">
         <v>24</v>
       </c>
       <c r="D194" s="1" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
     </row>
     <row r="195" spans="1:4">
@@ -6221,13 +6350,13 @@
         <v>8009</v>
       </c>
       <c r="B195" s="1" t="s">
+        <v>477</v>
+      </c>
+      <c r="C195" t="s">
+        <v>287</v>
+      </c>
+      <c r="D195" s="1" t="s">
         <v>478</v>
-      </c>
-      <c r="C195" t="s">
-        <v>288</v>
-      </c>
-      <c r="D195" s="1" t="s">
-        <v>479</v>
       </c>
     </row>
     <row r="196" spans="1:4">
@@ -6235,13 +6364,13 @@
         <v>8010</v>
       </c>
       <c r="B196" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="C196" t="s">
+        <v>287</v>
+      </c>
+      <c r="D196" s="1" t="s">
         <v>480</v>
-      </c>
-      <c r="C196" t="s">
-        <v>288</v>
-      </c>
-      <c r="D196" s="1" t="s">
-        <v>481</v>
       </c>
     </row>
     <row r="197" spans="1:4">
@@ -6249,13 +6378,13 @@
         <v>8011</v>
       </c>
       <c r="B197" s="1" t="s">
+        <v>481</v>
+      </c>
+      <c r="C197" t="s">
+        <v>287</v>
+      </c>
+      <c r="D197" s="1" t="s">
         <v>482</v>
-      </c>
-      <c r="C197" t="s">
-        <v>288</v>
-      </c>
-      <c r="D197" s="1" t="s">
-        <v>483</v>
       </c>
     </row>
     <row r="198" spans="1:4">
@@ -6263,13 +6392,13 @@
         <v>8012</v>
       </c>
       <c r="B198" s="1" t="s">
+        <v>483</v>
+      </c>
+      <c r="C198" t="s">
+        <v>21</v>
+      </c>
+      <c r="D198" s="1" t="s">
         <v>484</v>
-      </c>
-      <c r="C198" t="s">
-        <v>21</v>
-      </c>
-      <c r="D198" s="1" t="s">
-        <v>485</v>
       </c>
     </row>
     <row r="199" spans="1:4">
@@ -6277,13 +6406,13 @@
         <v>8013</v>
       </c>
       <c r="B199" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="C199" t="s">
+        <v>21</v>
+      </c>
+      <c r="D199" s="1" t="s">
         <v>486</v>
-      </c>
-      <c r="C199" t="s">
-        <v>21</v>
-      </c>
-      <c r="D199" s="1" t="s">
-        <v>487</v>
       </c>
     </row>
     <row r="200" spans="1:4">
@@ -6291,13 +6420,13 @@
         <v>8014</v>
       </c>
       <c r="B200" s="1" t="s">
+        <v>487</v>
+      </c>
+      <c r="C200" t="s">
+        <v>21</v>
+      </c>
+      <c r="D200" s="1" t="s">
         <v>488</v>
-      </c>
-      <c r="C200" t="s">
-        <v>21</v>
-      </c>
-      <c r="D200" s="1" t="s">
-        <v>489</v>
       </c>
     </row>
     <row r="201" spans="1:4">
@@ -6305,13 +6434,13 @@
         <v>8015</v>
       </c>
       <c r="B201" s="1" t="s">
+        <v>489</v>
+      </c>
+      <c r="C201" t="s">
+        <v>21</v>
+      </c>
+      <c r="D201" s="1" t="s">
         <v>490</v>
-      </c>
-      <c r="C201" t="s">
-        <v>21</v>
-      </c>
-      <c r="D201" s="1" t="s">
-        <v>491</v>
       </c>
     </row>
     <row r="202" spans="1:4">
@@ -6319,13 +6448,13 @@
         <v>8016</v>
       </c>
       <c r="B202" s="1" t="s">
+        <v>491</v>
+      </c>
+      <c r="C202" t="s">
+        <v>21</v>
+      </c>
+      <c r="D202" s="1" t="s">
         <v>492</v>
-      </c>
-      <c r="C202" t="s">
-        <v>21</v>
-      </c>
-      <c r="D202" s="1" t="s">
-        <v>493</v>
       </c>
     </row>
     <row r="203" spans="1:4">
@@ -6333,13 +6462,13 @@
         <v>8017</v>
       </c>
       <c r="B203" s="1" t="s">
+        <v>493</v>
+      </c>
+      <c r="C203" t="s">
+        <v>21</v>
+      </c>
+      <c r="D203" s="1" t="s">
         <v>494</v>
-      </c>
-      <c r="C203" t="s">
-        <v>21</v>
-      </c>
-      <c r="D203" s="1" t="s">
-        <v>495</v>
       </c>
     </row>
   </sheetData>

</xml_diff>